<commit_message>
E-book Excel : chapitre 4 (tableaux croisés et graphiques vérifiés, 75 contrôles)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T8L22svZaEaGYSwza4q3Yc
</commit_message>
<xml_diff>
--- a/produits/preuves/sortie/c1-texte-valeur/c1-texte-valeur.xlsx
+++ b/produits/preuves/sortie/c1-texte-valeur/c1-texte-valeur.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t xml:space="preserve">Article</t>
   </si>
@@ -48,6 +48,9 @@
   </si>
   <si>
     <t xml:space="preserve">IA 4o-mini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IA 5-mini</t>
   </si>
 </sst>
 </file>
@@ -254,7 +257,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.97"/>
@@ -327,6 +330,15 @@
         <v>#VALUE!</v>
       </c>
     </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="0" t="e">
+        <f aca="false">valeur(SUBSTITUTE(B2," F",""))</f>
+        <v>#NAME?</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>